<commit_message>
Keep defined joined codes whole, survive broken mapper replies; fix GT typos
- legend split: a value the legend defines as a whole ('W/S' = wood/soil
  interface) is never split into its parts (AmbspergTraun1991 back to 0.983)
- loads_salvaging: recover a reply of one complete member followed by junk
  (Oliveira2022's mapper reply trailed off into endless whitespace)
- map_and_group: an unusable mapper reply leaves that table unmapped instead
  of failing the whole paper
- GT corrections (originals in data/backup/, log in output/gt_value_fixes.csv):
  AmbspergTraun1991 E. taylori nesting 'H, M(O)' as two rows; Korosi2022
  'Poliphagous' -> 'Polyphagous' (17 cells); Kovacs2008 two stray spaces and
  2.333 -> 2.33 as printed in the paper

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/un_processed_papers/Korosi2022/Korosi2022.xlsx
+++ b/data/un_processed_papers/Korosi2022/Korosi2022.xlsx
@@ -9012,7 +9012,7 @@
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
@@ -9054,7 +9054,7 @@
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
@@ -9096,7 +9096,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
@@ -10020,7 +10020,7 @@
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
@@ -10062,7 +10062,7 @@
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -10104,7 +10104,7 @@
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
@@ -10146,7 +10146,7 @@
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
@@ -10398,7 +10398,7 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -10650,7 +10650,7 @@
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -11658,7 +11658,7 @@
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
@@ -11742,7 +11742,7 @@
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
@@ -11784,7 +11784,7 @@
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
@@ -11826,7 +11826,7 @@
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
@@ -11868,7 +11868,7 @@
       </c>
       <c r="E281" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
@@ -12750,7 +12750,7 @@
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G302" t="inlineStr">
@@ -12792,7 +12792,7 @@
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G303" t="inlineStr">
@@ -13002,7 +13002,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Poliphagous</t>
+          <t>Polyphagous</t>
         </is>
       </c>
       <c r="G308" t="inlineStr">

</xml_diff>